<commit_message>
Update translation on all forms to just be `en`
</commit_message>
<xml_diff>
--- a/basic-forms/forms/app/select_contact.xlsx
+++ b/basic-forms/forms/app/select_contact.xlsx
@@ -426,7 +426,7 @@
     <t xml:space="preserve">name</t>
   </si>
   <si>
-    <t xml:space="preserve">label::English (en)</t>
+    <t xml:space="preserve">label::en</t>
   </si>
   <si>
     <t xml:space="preserve">relevant</t>
@@ -740,20 +740,24 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1706,7 +1710,7 @@
       </c>
       <c r="B2" s="1" t="str">
         <f aca="true">TEXT(NOW(), "yyyymmddhhmmss")</f>
-        <v>20260618173626</v>
+        <v>20260722163919</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>49</v>
@@ -1770,160 +1774,160 @@
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="4" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="4" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="4" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="4" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="4" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="4" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="4" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="4" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="4" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="4" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="4" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="4" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="A13" s="4" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="A14" s="4" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+      <c r="A15" s="4" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+      <c r="A16" s="4" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="A17" s="4" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+      <c r="A18" s="4" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+      <c r="A19" s="4" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+      <c r="A20" s="4" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+      <c r="A21" s="4" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
+      <c r="A22" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
+      <c r="A23" s="4" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
+      <c r="A24" s="4" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
+      <c r="A25" s="4" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="s">
+      <c r="A26" s="4" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="s">
+      <c r="A27" s="4" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="s">
+      <c r="A28" s="4" t="s">
         <v>74</v>
       </c>
     </row>

</xml_diff>